<commit_message>
adapted labeling of preprocessing and vemamodelling in py and csv, xls
</commit_message>
<xml_diff>
--- a/IMAGE-Mat/input/vehicles/data_raw/battery_weights_kg.xlsx
+++ b/IMAGE-Mat/input/vehicles/data_raw/battery_weights_kg.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="23328"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27928"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\surfdrive\Paper_5\Vehicle_Material_Model_Dynamic\vehicle_data\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Admin\surfdrive - Sebastiaan Deetman@surfdrive.surf.nl\Github\Image\image-materials\IMAGE-Mat\input\vehicles\data_raw\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9000425D-DC68-45E6-B8E4-1153DCCE4257}" xr6:coauthVersionLast="45" xr6:coauthVersionMax="45" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B95BB87D-898A-4ED8-B57F-DDCF14F8859C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="13320" windowHeight="15600" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="battery_weights_kg_original" sheetId="2" r:id="rId1"/>
@@ -21,7 +21,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="20">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="71" uniqueCount="26">
   <si>
     <t>kg</t>
   </si>
@@ -81,6 +81,24 @@
   </si>
   <si>
     <t>kWh/kg</t>
+  </si>
+  <si>
+    <t>Light Commercial Vehicles</t>
+  </si>
+  <si>
+    <t>Medium Freight Trucks</t>
+  </si>
+  <si>
+    <t>Heavy Freight Trucks</t>
+  </si>
+  <si>
+    <t>Midi Buses</t>
+  </si>
+  <si>
+    <t>Regular Buses</t>
+  </si>
+  <si>
+    <t>Cars</t>
   </si>
 </sst>
 </file>
@@ -1724,22 +1742,22 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
-        <v>2</v>
+        <v>20</v>
       </c>
       <c r="D1" t="s">
-        <v>3</v>
+        <v>21</v>
       </c>
       <c r="E1" t="s">
-        <v>4</v>
+        <v>22</v>
       </c>
       <c r="F1" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
       <c r="G1" t="s">
-        <v>6</v>
+        <v>24</v>
       </c>
       <c r="H1" t="s">
-        <v>7</v>
+        <v>25</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">

</xml_diff>